<commit_message>
Update TU_test: add bash runner, update requirements
</commit_message>
<xml_diff>
--- a/TU_test/TestData/Login_TestCases.xlsx
+++ b/TU_test/TestData/Login_TestCases.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>6.06 sec</t>
+          <t>6.18 sec</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr"/>
@@ -711,7 +711,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>5.2 sec</t>
+          <t>5.15 sec</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr"/>
@@ -765,7 +765,7 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>4.58 sec</t>
+          <t>4.62 sec</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>3.41 sec</t>
+          <t>3.21 sec</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr"/>
@@ -873,7 +873,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>5.4 sec</t>
+          <t>5.55 sec</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
@@ -927,7 +927,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>0.14 sec</t>
+          <t>0.01 sec</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>1.15 sec</t>
+          <t>1.17 sec</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr"/>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>0.91 sec</t>
+          <t>0.92 sec</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr"/>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>0.49 sec</t>
+          <t>0.4 sec</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>0.02 sec</t>
+          <t>0.01 sec</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr"/>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>0.5 sec</t>
+          <t>0.51 sec</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>3.76 sec</t>
+          <t>3.78 sec</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>2.12</v>
+        <v>0.58</v>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="n"/>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="4" t="n"/>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>1.46</v>
+        <v>0.67</v>
       </c>
       <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="n"/>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>2.13</v>
+        <v>1.03</v>
       </c>
       <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="4" t="n"/>
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>1.74</v>
+        <v>1.11</v>
       </c>
       <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="4" t="n"/>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>2.52 sec</t>
+          <t>2.55 sec</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr"/>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>0.71 sec</t>
+          <t>0.7 sec</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr"/>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>0.72 sec</t>
+          <t>0.69 sec</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr"/>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>0.7 sec</t>
+          <t>0.66 sec</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>0.77 sec</t>
+          <t>0.7 sec</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr"/>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>2.41 sec</t>
+          <t>2.37 sec</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr"/>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>1.57 sec</t>
+          <t>1.45 sec</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr"/>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>0.01 sec</t>
+          <t>0.02 sec</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr"/>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>3.51 sec</t>
+          <t>3.39 sec</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr"/>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>0.77 sec</t>
+          <t>0.72 sec</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr"/>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>0.74 sec</t>
+          <t>0.77 sec</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr"/>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>0.72 sec</t>
+          <t>0.78 sec</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr"/>

</xml_diff>